<commit_message>
Support up to 25 invoices and remove unused sheets (#283)
</commit_message>
<xml_diff>
--- a/src/excel_templates/expense_report_template.xlsx
+++ b/src/excel_templates/expense_report_template.xlsx
@@ -1,25 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11012"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rajpandya/workspace/purchase-request-site/purchase_request_site/excel_templates/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rajpandya/workspace/purchase-request-site/src/excel_templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB70C285-0CB3-EB40-B814-74EEFF7924DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54E68F8F-A26A-A946-88CE-51926A0B5163}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-41120" yWindow="-1380" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -30,9 +27,6 @@
         <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
-    </ext>
-    <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="acbvb7pwVcDa2U0pbs+Ftk9Ry4ZyHPZ9qNrw2HYqQqA="/>
     </ext>
   </extLst>
 </workbook>
@@ -115,7 +109,7 @@
     <numFmt numFmtId="164" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
     <numFmt numFmtId="165" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@"/>
   </numFmts>
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -177,18 +171,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="8"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
@@ -222,7 +204,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -278,21 +260,6 @@
     </border>
     <border>
       <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
         <color rgb="FF000000"/>
       </left>
       <right/>
@@ -333,30 +300,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right/>
       <top/>
@@ -380,7 +323,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -396,15 +339,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="17" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="165" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -416,9 +350,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="2" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -454,67 +385,48 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="17" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="17" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="17" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="17" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="12" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="10" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -538,22 +450,22 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>85396</xdr:colOff>
-      <xdr:row>18</xdr:row>
-      <xdr:rowOff>79473</xdr:rowOff>
+      <xdr:colOff>59120</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>61957</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>275239</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>232540</xdr:rowOff>
+      <xdr:colOff>248963</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>49486</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9FF2CA13-4754-9861-F7EB-F315CBC6AABA}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -562,13 +474,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
         <a:srcRect/>
         <a:stretch>
           <a:fillRect/>
@@ -576,22 +482,16 @@
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="4276396" y="3817214"/>
-          <a:ext cx="925567" cy="639171"/>
+          <a:off x="4841327" y="6499543"/>
+          <a:ext cx="1030670" cy="513046"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
         <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
@@ -599,9 +499,9 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>157655</xdr:colOff>
-      <xdr:row>18</xdr:row>
-      <xdr:rowOff>164224</xdr:rowOff>
+      <xdr:colOff>43793</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>85397</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="781050" cy="571500"/>
     <xdr:pic>
@@ -609,7 +509,7 @@
         <xdr:cNvPr id="3" name="Image 2" descr="Picture">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5591E8DB-209D-4CB0-825D-98EC3A7D85CC}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000003000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -623,7 +523,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5820103" y="3901965"/>
+          <a:off x="6507655" y="6522983"/>
           <a:ext cx="781050" cy="571500"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -850,66 +750,66 @@
     <col min="9" max="26" width="8.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="24" x14ac:dyDescent="0.3">
-      <c r="A1" s="51" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="52"/>
-      <c r="C1" s="52"/>
-      <c r="D1" s="52"/>
-      <c r="E1" s="52"/>
-      <c r="F1" s="52"/>
-      <c r="G1" s="52"/>
+    <row r="1" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="41" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="42"/>
+      <c r="C1" s="42"/>
+      <c r="D1" s="42"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="42"/>
+      <c r="G1" s="42"/>
     </row>
     <row r="2" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="50"/>
+      <c r="C2" s="40"/>
       <c r="E2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="46"/>
-      <c r="G2" s="48"/>
+      <c r="F2" s="36"/>
+      <c r="G2" s="38"/>
     </row>
     <row r="3" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="47"/>
+      <c r="C3" s="37"/>
       <c r="D3" s="3"/>
       <c r="E3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F3" s="47"/>
-      <c r="G3" s="49"/>
+      <c r="F3" s="37"/>
+      <c r="G3" s="39"/>
     </row>
     <row r="4" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F4" s="45"/>
-    </row>
-    <row r="5" spans="1:14" ht="34" x14ac:dyDescent="0.2">
+      <c r="F4" s="35"/>
+    </row>
+    <row r="5" spans="1:14" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="33" t="s">
+      <c r="B5" s="26" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="34" t="s">
+      <c r="C5" s="27" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="37" t="s">
+      <c r="D5" s="28" t="s">
         <v>8</v>
       </c>
-      <c r="E5" s="37" t="s">
+      <c r="E5" s="28" t="s">
         <v>9</v>
       </c>
-      <c r="F5" s="37" t="s">
+      <c r="F5" s="28" t="s">
         <v>10</v>
       </c>
-      <c r="G5" s="38" t="s">
+      <c r="G5" s="29" t="s">
         <v>11</v>
       </c>
-      <c r="H5" s="37" t="s">
+      <c r="H5" s="28" t="s">
         <v>12</v>
       </c>
       <c r="I5" s="5"/>
@@ -920,427 +820,862 @@
       <c r="N5" s="5"/>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A6" s="32">
+      <c r="A6" s="25">
         <v>1</v>
       </c>
-      <c r="B6" s="42"/>
-      <c r="C6" s="43"/>
-      <c r="D6" s="40">
-        <v>0</v>
-      </c>
-      <c r="E6" s="40">
-        <v>0</v>
-      </c>
-      <c r="F6" s="40">
-        <v>0</v>
-      </c>
-      <c r="G6" s="41">
-        <f>F6+H6</f>
-        <v>0</v>
-      </c>
-      <c r="H6" s="10">
-        <f>0.13*F6</f>
-        <v>0</v>
-      </c>
-      <c r="I6" s="12"/>
-      <c r="J6" s="13"/>
-      <c r="K6" s="12"/>
-      <c r="L6" s="12"/>
-      <c r="M6" s="12"/>
-      <c r="N6" s="12"/>
-    </row>
-    <row r="7" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="32">
+      <c r="B6" s="32"/>
+      <c r="C6" s="33"/>
+      <c r="D6" s="30">
+        <v>0</v>
+      </c>
+      <c r="E6" s="30">
+        <v>0</v>
+      </c>
+      <c r="F6" s="30">
+        <v>0</v>
+      </c>
+      <c r="G6" s="31">
+        <f t="shared" ref="G6:G30" si="0">F6+H6</f>
+        <v>0</v>
+      </c>
+      <c r="H6" s="7">
+        <f t="shared" ref="H6:H30" si="1">0.13*F6</f>
+        <v>0</v>
+      </c>
+      <c r="I6" s="9"/>
+      <c r="J6" s="10"/>
+      <c r="K6" s="9"/>
+      <c r="L6" s="9"/>
+      <c r="M6" s="9"/>
+      <c r="N6" s="9"/>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A7" s="25">
         <v>2</v>
       </c>
-      <c r="B7" s="54"/>
-      <c r="C7" s="31"/>
-      <c r="D7" s="39">
-        <v>0</v>
-      </c>
-      <c r="E7" s="39">
-        <v>0</v>
-      </c>
-      <c r="F7" s="39">
-        <v>0</v>
-      </c>
-      <c r="G7" s="41">
-        <f t="shared" ref="G7:G10" si="0">F7+H7</f>
-        <v>0</v>
-      </c>
-      <c r="H7" s="10">
-        <f t="shared" ref="H7:H12" si="1">0.13*F7</f>
-        <v>0</v>
-      </c>
-      <c r="I7" s="12"/>
-      <c r="J7" s="12"/>
-      <c r="K7" s="12"/>
-      <c r="L7" s="12"/>
-      <c r="M7" s="12"/>
-      <c r="N7" s="12"/>
+      <c r="B7" s="32"/>
+      <c r="C7" s="33"/>
+      <c r="D7" s="30">
+        <v>0</v>
+      </c>
+      <c r="E7" s="30">
+        <v>0</v>
+      </c>
+      <c r="F7" s="30">
+        <v>0</v>
+      </c>
+      <c r="G7" s="31">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H7" s="7">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="I7" s="9"/>
+      <c r="J7" s="10"/>
+      <c r="K7" s="9"/>
+      <c r="L7" s="9"/>
+      <c r="M7" s="9"/>
+      <c r="N7" s="9"/>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A8" s="32">
+      <c r="A8" s="25">
         <v>3</v>
       </c>
-      <c r="B8" s="42"/>
-      <c r="C8" s="43"/>
-      <c r="D8" s="10">
-        <v>0</v>
-      </c>
-      <c r="E8" s="10">
-        <v>0</v>
-      </c>
-      <c r="F8" s="10">
-        <v>0</v>
-      </c>
-      <c r="G8" s="41">
+      <c r="B8" s="32"/>
+      <c r="C8" s="33"/>
+      <c r="D8" s="30">
+        <v>0</v>
+      </c>
+      <c r="E8" s="30">
+        <v>0</v>
+      </c>
+      <c r="F8" s="30">
+        <v>0</v>
+      </c>
+      <c r="G8" s="31">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H8" s="10">
+      <c r="H8" s="7">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="I8" s="12"/>
-      <c r="J8" s="12"/>
-      <c r="K8" s="12"/>
-      <c r="L8" s="12"/>
-      <c r="M8" s="12"/>
-      <c r="N8" s="12"/>
-    </row>
-    <row r="9" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="32">
+      <c r="I8" s="9"/>
+      <c r="J8" s="10"/>
+      <c r="K8" s="9"/>
+      <c r="L8" s="9"/>
+      <c r="M8" s="9"/>
+      <c r="N8" s="9"/>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A9" s="25">
         <v>4</v>
       </c>
-      <c r="B9" s="54"/>
-      <c r="C9" s="31"/>
-      <c r="D9" s="39">
-        <v>0</v>
-      </c>
-      <c r="E9" s="39">
-        <v>0</v>
-      </c>
-      <c r="F9" s="39">
-        <v>0</v>
-      </c>
-      <c r="G9" s="41">
+      <c r="B9" s="32"/>
+      <c r="C9" s="33"/>
+      <c r="D9" s="30">
+        <v>0</v>
+      </c>
+      <c r="E9" s="30">
+        <v>0</v>
+      </c>
+      <c r="F9" s="30">
+        <v>0</v>
+      </c>
+      <c r="G9" s="31">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H9" s="10">
+      <c r="H9" s="7">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="I9" s="12"/>
-      <c r="J9" s="12"/>
-      <c r="K9" s="12"/>
-      <c r="L9" s="12"/>
-      <c r="M9" s="12"/>
-      <c r="N9" s="12"/>
-    </row>
-    <row r="10" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="32">
+      <c r="I9" s="9"/>
+      <c r="J9" s="10"/>
+      <c r="K9" s="9"/>
+      <c r="L9" s="9"/>
+      <c r="M9" s="9"/>
+      <c r="N9" s="9"/>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A10" s="25">
         <v>5</v>
       </c>
-      <c r="B10" s="42"/>
-      <c r="C10" s="43"/>
-      <c r="D10" s="10">
-        <v>0</v>
-      </c>
-      <c r="E10" s="10">
-        <v>0</v>
-      </c>
-      <c r="F10" s="10">
-        <v>0</v>
-      </c>
-      <c r="G10" s="41">
+      <c r="B10" s="32"/>
+      <c r="C10" s="33"/>
+      <c r="D10" s="30">
+        <v>0</v>
+      </c>
+      <c r="E10" s="30">
+        <v>0</v>
+      </c>
+      <c r="F10" s="30">
+        <v>0</v>
+      </c>
+      <c r="G10" s="31">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H10" s="10">
+      <c r="H10" s="7">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="I10" s="12"/>
-      <c r="J10" s="12"/>
-      <c r="K10" s="12"/>
-      <c r="L10" s="12"/>
-      <c r="M10" s="12"/>
-      <c r="N10" s="12"/>
-    </row>
-    <row r="11" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="7">
+      <c r="I10" s="9"/>
+      <c r="J10" s="10"/>
+      <c r="K10" s="9"/>
+      <c r="L10" s="9"/>
+      <c r="M10" s="9"/>
+      <c r="N10" s="9"/>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A11" s="25">
         <v>6</v>
       </c>
-      <c r="B11" s="35"/>
-      <c r="C11" s="36"/>
-      <c r="D11" s="39">
-        <v>0</v>
-      </c>
-      <c r="E11" s="39">
-        <v>0</v>
-      </c>
-      <c r="F11" s="39">
-        <v>0</v>
-      </c>
-      <c r="G11" s="41">
-        <f t="shared" ref="G11:G15" si="2">F11+H11</f>
-        <v>0</v>
-      </c>
-      <c r="H11" s="10">
+      <c r="B11" s="32"/>
+      <c r="C11" s="33"/>
+      <c r="D11" s="30">
+        <v>0</v>
+      </c>
+      <c r="E11" s="30">
+        <v>0</v>
+      </c>
+      <c r="F11" s="30">
+        <v>0</v>
+      </c>
+      <c r="G11" s="31">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H11" s="7">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="I11" s="12"/>
-      <c r="J11" s="12"/>
-      <c r="K11" s="12"/>
-      <c r="L11" s="12"/>
-      <c r="M11" s="12"/>
-      <c r="N11" s="12"/>
-    </row>
-    <row r="12" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="7">
+      <c r="I11" s="9"/>
+      <c r="J11" s="10"/>
+      <c r="K11" s="9"/>
+      <c r="L11" s="9"/>
+      <c r="M11" s="9"/>
+      <c r="N11" s="9"/>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A12" s="25">
         <v>7</v>
       </c>
-      <c r="B12" s="29"/>
-      <c r="C12" s="30"/>
-      <c r="D12" s="10">
-        <v>0</v>
-      </c>
-      <c r="E12" s="10">
-        <v>0</v>
-      </c>
-      <c r="F12" s="10">
-        <v>0</v>
-      </c>
-      <c r="G12" s="41">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="H12" s="10">
+      <c r="B12" s="32"/>
+      <c r="C12" s="33"/>
+      <c r="D12" s="30">
+        <v>0</v>
+      </c>
+      <c r="E12" s="30">
+        <v>0</v>
+      </c>
+      <c r="F12" s="30">
+        <v>0</v>
+      </c>
+      <c r="G12" s="31">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H12" s="7">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="I12" s="12"/>
-      <c r="J12" s="12"/>
-      <c r="K12" s="12"/>
-      <c r="L12" s="12"/>
-      <c r="M12" s="12"/>
-      <c r="N12" s="12"/>
-    </row>
-    <row r="13" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="7">
+      <c r="I12" s="9"/>
+      <c r="J12" s="10"/>
+      <c r="K12" s="9"/>
+      <c r="L12" s="9"/>
+      <c r="M12" s="9"/>
+      <c r="N12" s="9"/>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A13" s="25">
         <v>8</v>
       </c>
-      <c r="B13" s="29"/>
-      <c r="C13" s="30"/>
-      <c r="D13" s="10">
-        <v>0</v>
-      </c>
-      <c r="E13" s="10">
-        <v>0</v>
-      </c>
-      <c r="F13" s="10">
-        <v>0</v>
-      </c>
-      <c r="G13" s="41">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="H13" s="10">
-        <f t="shared" ref="H13:H15" si="3">0.13*F13</f>
-        <v>0</v>
-      </c>
-      <c r="I13" s="12"/>
-      <c r="J13" s="12"/>
-      <c r="K13" s="12"/>
-      <c r="L13" s="12"/>
-      <c r="M13" s="12"/>
-      <c r="N13" s="12"/>
-    </row>
-    <row r="14" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="7">
+      <c r="B13" s="32"/>
+      <c r="C13" s="33"/>
+      <c r="D13" s="30">
+        <v>0</v>
+      </c>
+      <c r="E13" s="30">
+        <v>0</v>
+      </c>
+      <c r="F13" s="30">
+        <v>0</v>
+      </c>
+      <c r="G13" s="31">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H13" s="7">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="I13" s="9"/>
+      <c r="J13" s="10"/>
+      <c r="K13" s="9"/>
+      <c r="L13" s="9"/>
+      <c r="M13" s="9"/>
+      <c r="N13" s="9"/>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A14" s="25">
         <v>9</v>
       </c>
-      <c r="B14" s="8"/>
-      <c r="C14" s="9"/>
-      <c r="D14" s="10">
-        <v>0</v>
-      </c>
-      <c r="E14" s="10">
-        <v>0</v>
-      </c>
-      <c r="F14" s="10">
-        <v>0</v>
-      </c>
-      <c r="G14" s="41">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="H14" s="10">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="I14" s="12"/>
-      <c r="J14" s="12"/>
-      <c r="K14" s="12"/>
-      <c r="L14" s="12"/>
-      <c r="M14" s="12"/>
-      <c r="N14" s="12"/>
-    </row>
-    <row r="15" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="7">
+      <c r="B14" s="32"/>
+      <c r="C14" s="33"/>
+      <c r="D14" s="30">
+        <v>0</v>
+      </c>
+      <c r="E14" s="30">
+        <v>0</v>
+      </c>
+      <c r="F14" s="30">
+        <v>0</v>
+      </c>
+      <c r="G14" s="31">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H14" s="7">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="I14" s="9"/>
+      <c r="J14" s="10"/>
+      <c r="K14" s="9"/>
+      <c r="L14" s="9"/>
+      <c r="M14" s="9"/>
+      <c r="N14" s="9"/>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A15" s="25">
         <v>10</v>
       </c>
-      <c r="B15" s="14"/>
-      <c r="C15" s="9"/>
-      <c r="D15" s="10">
-        <v>0</v>
-      </c>
-      <c r="E15" s="10">
-        <v>0</v>
-      </c>
-      <c r="F15" s="10">
-        <v>0</v>
-      </c>
-      <c r="G15" s="41">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="H15" s="10">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="I15" s="12"/>
-      <c r="J15" s="12"/>
-      <c r="K15" s="12"/>
-      <c r="L15" s="12"/>
-      <c r="M15" s="12"/>
-      <c r="N15" s="12"/>
-    </row>
-    <row r="16" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="15" t="s">
+      <c r="B15" s="32"/>
+      <c r="C15" s="33"/>
+      <c r="D15" s="30">
+        <v>0</v>
+      </c>
+      <c r="E15" s="30">
+        <v>0</v>
+      </c>
+      <c r="F15" s="30">
+        <v>0</v>
+      </c>
+      <c r="G15" s="31">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H15" s="7">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="I15" s="9"/>
+      <c r="J15" s="10"/>
+      <c r="K15" s="9"/>
+      <c r="L15" s="9"/>
+      <c r="M15" s="9"/>
+      <c r="N15" s="9"/>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A16" s="25">
+        <v>11</v>
+      </c>
+      <c r="B16" s="32"/>
+      <c r="C16" s="33"/>
+      <c r="D16" s="30">
+        <v>0</v>
+      </c>
+      <c r="E16" s="30">
+        <v>0</v>
+      </c>
+      <c r="F16" s="30">
+        <v>0</v>
+      </c>
+      <c r="G16" s="31">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H16" s="7">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="I16" s="9"/>
+      <c r="J16" s="10"/>
+      <c r="K16" s="9"/>
+      <c r="L16" s="9"/>
+      <c r="M16" s="9"/>
+      <c r="N16" s="9"/>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A17" s="25">
+        <v>12</v>
+      </c>
+      <c r="B17" s="32"/>
+      <c r="C17" s="33"/>
+      <c r="D17" s="30">
+        <v>0</v>
+      </c>
+      <c r="E17" s="30">
+        <v>0</v>
+      </c>
+      <c r="F17" s="30">
+        <v>0</v>
+      </c>
+      <c r="G17" s="31">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H17" s="7">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="I17" s="9"/>
+      <c r="J17" s="10"/>
+      <c r="K17" s="9"/>
+      <c r="L17" s="9"/>
+      <c r="M17" s="9"/>
+      <c r="N17" s="9"/>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A18" s="25">
         <v>13</v>
       </c>
-      <c r="B16" s="16"/>
-      <c r="C16" s="17"/>
-      <c r="D16" s="18">
-        <f>SUM(D6:D15)</f>
-        <v>0</v>
-      </c>
-      <c r="E16" s="18">
-        <f>SUM(E6:E15)</f>
-        <v>0</v>
-      </c>
-      <c r="F16" s="18">
-        <f>SUM(F6:F15)</f>
-        <v>0</v>
-      </c>
-      <c r="G16" s="11">
-        <f>SUM(G6:G15)</f>
-        <v>0</v>
-      </c>
-      <c r="H16" s="18">
-        <f>SUM(H6:H15)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="19"/>
-      <c r="B17" s="20"/>
-      <c r="D17" s="21"/>
-      <c r="F17" s="22" t="s">
+      <c r="B18" s="32"/>
+      <c r="C18" s="33"/>
+      <c r="D18" s="30">
+        <v>0</v>
+      </c>
+      <c r="E18" s="30">
+        <v>0</v>
+      </c>
+      <c r="F18" s="30">
+        <v>0</v>
+      </c>
+      <c r="G18" s="31">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H18" s="7">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="I18" s="9"/>
+      <c r="J18" s="10"/>
+      <c r="K18" s="9"/>
+      <c r="L18" s="9"/>
+      <c r="M18" s="9"/>
+      <c r="N18" s="9"/>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A19" s="25">
         <v>14</v>
       </c>
-      <c r="G17" s="23">
-        <f>G16</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="19" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="20" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="44"/>
-    </row>
-    <row r="21" spans="1:14" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="2"/>
-      <c r="B21" s="2"/>
-      <c r="D21" s="24"/>
-      <c r="F21" s="24"/>
-    </row>
-    <row r="22" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="25" t="s">
+      <c r="B19" s="32"/>
+      <c r="C19" s="33"/>
+      <c r="D19" s="30">
+        <v>0</v>
+      </c>
+      <c r="E19" s="30">
+        <v>0</v>
+      </c>
+      <c r="F19" s="30">
+        <v>0</v>
+      </c>
+      <c r="G19" s="31">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H19" s="7">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="I19" s="9"/>
+      <c r="J19" s="10"/>
+      <c r="K19" s="9"/>
+      <c r="L19" s="9"/>
+      <c r="M19" s="9"/>
+      <c r="N19" s="9"/>
+    </row>
+    <row r="20" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A20" s="25">
         <v>15</v>
       </c>
-      <c r="D22" s="26" t="s">
+      <c r="B20" s="32"/>
+      <c r="C20" s="33"/>
+      <c r="D20" s="30">
+        <v>0</v>
+      </c>
+      <c r="E20" s="30">
+        <v>0</v>
+      </c>
+      <c r="F20" s="30">
+        <v>0</v>
+      </c>
+      <c r="G20" s="31">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H20" s="7">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="I20" s="9"/>
+      <c r="J20" s="10"/>
+      <c r="K20" s="9"/>
+      <c r="L20" s="9"/>
+      <c r="M20" s="9"/>
+      <c r="N20" s="9"/>
+    </row>
+    <row r="21" spans="1:14" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="25">
         <v>16</v>
       </c>
-      <c r="E22" s="26" t="s">
+      <c r="B21" s="32"/>
+      <c r="C21" s="33"/>
+      <c r="D21" s="30">
+        <v>0</v>
+      </c>
+      <c r="E21" s="30">
+        <v>0</v>
+      </c>
+      <c r="F21" s="30">
+        <v>0</v>
+      </c>
+      <c r="G21" s="31">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H21" s="7">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="I21" s="9"/>
+      <c r="J21" s="10"/>
+      <c r="K21" s="9"/>
+      <c r="L21" s="9"/>
+      <c r="M21" s="9"/>
+      <c r="N21" s="9"/>
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A22" s="25">
         <v>17</v>
       </c>
-      <c r="F22" s="26"/>
-      <c r="G22" s="26"/>
-    </row>
-    <row r="23" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="D23" s="24"/>
-      <c r="E23" s="24" t="s">
+      <c r="B22" s="32"/>
+      <c r="C22" s="33"/>
+      <c r="D22" s="30">
+        <v>0</v>
+      </c>
+      <c r="E22" s="30">
+        <v>0</v>
+      </c>
+      <c r="F22" s="30">
+        <v>0</v>
+      </c>
+      <c r="G22" s="31">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H22" s="7">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="I22" s="9"/>
+      <c r="J22" s="10"/>
+      <c r="K22" s="9"/>
+      <c r="L22" s="9"/>
+      <c r="M22" s="9"/>
+      <c r="N22" s="9"/>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A23" s="25">
         <v>18</v>
       </c>
-      <c r="F23" s="24"/>
-      <c r="G23" s="24"/>
-    </row>
-    <row r="24" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="25" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="G25" s="27"/>
-      <c r="H25" s="28"/>
-      <c r="I25" s="28"/>
-      <c r="J25" s="28"/>
-      <c r="K25" s="28"/>
-      <c r="L25" s="28"/>
-      <c r="M25" s="28"/>
-      <c r="N25" s="28"/>
-    </row>
-    <row r="26" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="25" t="s">
+      <c r="B23" s="32"/>
+      <c r="C23" s="33"/>
+      <c r="D23" s="30">
+        <v>0</v>
+      </c>
+      <c r="E23" s="30">
+        <v>0</v>
+      </c>
+      <c r="F23" s="30">
+        <v>0</v>
+      </c>
+      <c r="G23" s="31">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H23" s="7">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="I23" s="9"/>
+      <c r="J23" s="10"/>
+      <c r="K23" s="9"/>
+      <c r="L23" s="9"/>
+      <c r="M23" s="9"/>
+      <c r="N23" s="9"/>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A24" s="25">
         <v>19</v>
       </c>
-    </row>
-    <row r="27" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="53" t="s">
+      <c r="B24" s="32"/>
+      <c r="C24" s="33"/>
+      <c r="D24" s="30">
+        <v>0</v>
+      </c>
+      <c r="E24" s="30">
+        <v>0</v>
+      </c>
+      <c r="F24" s="30">
+        <v>0</v>
+      </c>
+      <c r="G24" s="31">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H24" s="7">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="I24" s="9"/>
+      <c r="J24" s="10"/>
+      <c r="K24" s="9"/>
+      <c r="L24" s="9"/>
+      <c r="M24" s="9"/>
+      <c r="N24" s="9"/>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A25" s="25">
         <v>20</v>
       </c>
-      <c r="B27" s="52"/>
-      <c r="C27" s="52"/>
-      <c r="D27" s="52"/>
-      <c r="E27" s="52"/>
-      <c r="F27" s="52"/>
-    </row>
-    <row r="28" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="3" t="s">
+      <c r="B25" s="32"/>
+      <c r="C25" s="33"/>
+      <c r="D25" s="30">
+        <v>0</v>
+      </c>
+      <c r="E25" s="30">
+        <v>0</v>
+      </c>
+      <c r="F25" s="30">
+        <v>0</v>
+      </c>
+      <c r="G25" s="31">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H25" s="7">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="I25" s="9"/>
+      <c r="J25" s="10"/>
+      <c r="K25" s="9"/>
+      <c r="L25" s="9"/>
+      <c r="M25" s="9"/>
+      <c r="N25" s="9"/>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A26" s="25">
         <v>21</v>
       </c>
-    </row>
-    <row r="29" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="30" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="31" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="32" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="33" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="34" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="35" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="36" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="37" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="38" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="39" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="40" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="41" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="42" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="43" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="44" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="45" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="46" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="47" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="48" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+      <c r="B26" s="32"/>
+      <c r="C26" s="33"/>
+      <c r="D26" s="30">
+        <v>0</v>
+      </c>
+      <c r="E26" s="30">
+        <v>0</v>
+      </c>
+      <c r="F26" s="30">
+        <v>0</v>
+      </c>
+      <c r="G26" s="31">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H26" s="7">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="I26" s="9"/>
+      <c r="J26" s="10"/>
+      <c r="K26" s="9"/>
+      <c r="L26" s="9"/>
+      <c r="M26" s="9"/>
+      <c r="N26" s="9"/>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A27" s="25">
+        <v>22</v>
+      </c>
+      <c r="B27" s="32"/>
+      <c r="C27" s="33"/>
+      <c r="D27" s="30">
+        <v>0</v>
+      </c>
+      <c r="E27" s="30">
+        <v>0</v>
+      </c>
+      <c r="F27" s="30">
+        <v>0</v>
+      </c>
+      <c r="G27" s="31">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H27" s="7">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="I27" s="9"/>
+      <c r="J27" s="10"/>
+      <c r="K27" s="9"/>
+      <c r="L27" s="9"/>
+      <c r="M27" s="9"/>
+      <c r="N27" s="9"/>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A28" s="25">
+        <v>23</v>
+      </c>
+      <c r="B28" s="32"/>
+      <c r="C28" s="33"/>
+      <c r="D28" s="30">
+        <v>0</v>
+      </c>
+      <c r="E28" s="30">
+        <v>0</v>
+      </c>
+      <c r="F28" s="30">
+        <v>0</v>
+      </c>
+      <c r="G28" s="31">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H28" s="7">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="I28" s="9"/>
+      <c r="J28" s="10"/>
+      <c r="K28" s="9"/>
+      <c r="L28" s="9"/>
+      <c r="M28" s="9"/>
+      <c r="N28" s="9"/>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A29" s="25">
+        <v>24</v>
+      </c>
+      <c r="B29" s="32"/>
+      <c r="C29" s="33"/>
+      <c r="D29" s="30">
+        <v>0</v>
+      </c>
+      <c r="E29" s="30">
+        <v>0</v>
+      </c>
+      <c r="F29" s="30">
+        <v>0</v>
+      </c>
+      <c r="G29" s="31">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H29" s="7">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="I29" s="9"/>
+      <c r="J29" s="10"/>
+      <c r="K29" s="9"/>
+      <c r="L29" s="9"/>
+      <c r="M29" s="9"/>
+      <c r="N29" s="9"/>
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A30" s="25">
+        <v>25</v>
+      </c>
+      <c r="B30" s="32"/>
+      <c r="C30" s="33"/>
+      <c r="D30" s="30">
+        <v>0</v>
+      </c>
+      <c r="E30" s="30">
+        <v>0</v>
+      </c>
+      <c r="F30" s="30">
+        <v>0</v>
+      </c>
+      <c r="G30" s="31">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H30" s="7">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="I30" s="9"/>
+      <c r="J30" s="10"/>
+      <c r="K30" s="9"/>
+      <c r="L30" s="9"/>
+      <c r="M30" s="9"/>
+      <c r="N30" s="9"/>
+    </row>
+    <row r="31" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A31" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="B31" s="12"/>
+      <c r="C31" s="13"/>
+      <c r="D31" s="14">
+        <f>SUM(D6:D30)</f>
+        <v>0</v>
+      </c>
+      <c r="E31" s="14">
+        <f>SUM(E6:E30)</f>
+        <v>0</v>
+      </c>
+      <c r="F31" s="14">
+        <f>SUM(F6:F30)</f>
+        <v>0</v>
+      </c>
+      <c r="G31" s="8">
+        <f>SUM(G6:G30)</f>
+        <v>0</v>
+      </c>
+      <c r="H31" s="14">
+        <f>SUM(H6:H30)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A32" s="15"/>
+      <c r="B32" s="16"/>
+      <c r="D32" s="17"/>
+      <c r="F32" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="G32" s="19">
+        <f>G31</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="34" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="35" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A35" s="34"/>
+    </row>
+    <row r="36" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A36" s="2"/>
+      <c r="B36" s="2"/>
+      <c r="D36" s="20"/>
+      <c r="F36" s="20"/>
+    </row>
+    <row r="37" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A37" s="21" t="s">
+        <v>15</v>
+      </c>
+      <c r="D37" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="E37" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="F37" s="22"/>
+      <c r="G37" s="22"/>
+    </row>
+    <row r="38" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D38" s="20"/>
+      <c r="E38" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="F38" s="20"/>
+      <c r="G38" s="20"/>
+    </row>
+    <row r="39" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="40" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G40" s="23"/>
+      <c r="H40" s="24"/>
+      <c r="I40" s="24"/>
+      <c r="J40" s="24"/>
+      <c r="K40" s="24"/>
+      <c r="L40" s="24"/>
+      <c r="M40" s="24"/>
+      <c r="N40" s="24"/>
+    </row>
+    <row r="41" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A41" s="21" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="42" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A42" s="43" t="s">
+        <v>20</v>
+      </c>
+      <c r="B42" s="42"/>
+      <c r="C42" s="42"/>
+      <c r="D42" s="42"/>
+      <c r="E42" s="42"/>
+      <c r="F42" s="42"/>
+    </row>
+    <row r="43" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A43" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="44" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="45" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="46" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="47" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="48" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="49" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="50" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="51" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -2296,265 +2631,13 @@
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A27:F27"/>
+    <mergeCell ref="A42:F42"/>
   </mergeCells>
-  <phoneticPr fontId="10" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="A28" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="A28" r:id="rId1" display="https://www.bankofcanada.ca/rates/exchange/currency-converter/" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
-  <pageSetup orientation="landscape" r:id="rId2"/>
-  <drawing r:id="rId3"/>
+  <pageSetup orientation="landscape"/>
+  <drawing r:id="rId2"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100351D1D23F4A58043BBE384EF1CC13A0B" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="551746a8f748353412c924590d0cc7bb">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="1a264f36-df5c-4c23-a2b7-7f3f30b83ede" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9757548110673be55767ddfdfb996e4e" ns2:_="">
-    <xsd:import namespace="1a264f36-df5c-4c23-a2b7-7f3f30b83ede"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="1a264f36-df5c-4c23-a2b7-7f3f30b83ede" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="11" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="12" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="13" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="14" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="15" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="17" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="a073764d-e844-48d8-8cbc-d63b9d952867" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="18" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="19" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1a264f36-df5c-4c23-a2b7-7f3f30b83ede">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BCEC3260-1CA7-4D88-8FD6-50B5E2D6434D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="1a264f36-df5c-4c23-a2b7-7f3f30b83ede"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{21E525EF-B04A-472D-A8C2-E7BAB8EF13D1}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="1a264f36-df5c-4c23-a2b7-7f3f30b83ede"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{05733098-B355-4893-B1C3-03693DC8BD5A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>